<commit_message>
Reposition CANDRON as a provider of Canadian-made electrical equipment
Rewrite manufacturer, in-house and 'our Toronto facility' claims across
the site, range data, project stories, resources and metadata. The
/manufacturing page becomes the Canadian-Made page (how we source,
inspect, witness tests and deliver).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/candron-rfq-bid-scorecard.xlsx
+++ b/public/downloads/candron-rfq-bid-scorecard.xlsx
@@ -770,7 +770,7 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Free resource from CANDRON Energy Inc. · switchgear, switchboards and transformers designed, built and tested in Toronto · candron.com · +1 (647) 616-2595</t>
+          <t>Free resource from CANDRON Energy Inc. · providers of Canadian-made switchgear, switchboards and transformers · candron.com · +1 (647) 616-2595</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Free resource from CANDRON Energy Inc. · switchgear, switchboards and transformers designed, built and tested in Toronto · candron.com · +1 (647) 616-2595</t>
+          <t>Free resource from CANDRON Energy Inc. · providers of Canadian-made switchgear, switchboards and transformers · candron.com · +1 (647) 616-2595</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Free resource from CANDRON Energy Inc. · switchgear, switchboards and transformers designed, built and tested in Toronto · candron.com · +1 (647) 616-2595</t>
+          <t>Free resource from CANDRON Energy Inc. · providers of Canadian-made switchgear, switchboards and transformers · candron.com · +1 (647) 616-2595</t>
         </is>
       </c>
     </row>
@@ -2337,7 +2337,7 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Free resource from CANDRON Energy Inc. · switchgear, switchboards and transformers designed, built and tested in Toronto · candron.com · +1 (647) 616-2595</t>
+          <t>Free resource from CANDRON Energy Inc. · providers of Canadian-made switchgear, switchboards and transformers · candron.com · +1 (647) 616-2595</t>
         </is>
       </c>
     </row>

</xml_diff>